<commit_message>
feat: Add Phase 5 strategic features (Excel Owners Statement, VA/QRIS, Fit-Out SIK PDF, WBP/LWBP tariffs, CSAT rating)
- Add multi-tab Excel export (.xlsx) on Owner Statement Wizard
- Add Virtual Account (BCA, Mandiri, BNI, BRI, Permata, CIMB) & QRIS generator on contracts & invoices
- Add Fit-Out Permit / Surat Izin Kerja (SIK) model, workflow, views, and printable QWeb PDF
- Add PLN B3/I3 peak/off-peak (WBP/LWBP) dual electricity tariffs and meter reading computation
- Add CSAT star rating & feedback submission on tenant maintenance portal
- Update SOP User Guide and UAT test cases (Total: 69 TCs)
</commit_message>
<xml_diff>
--- a/Rental Property Management - Odoo 19 Custom Addon/docs/UAT_Tracker_Custom_Modules.xlsx
+++ b/Rental Property Management - Odoo 19 Custom Addon/docs/UAT_Tracker_Custom_Modules.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4309,6 +4309,191 @@
       <c r="G95" t="inlineStr">
         <is>
           <t>Legal / BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>TC-65</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>rental_management_financial_report</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Ekspor Excel (.xlsx) Laporan Pemilik</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Buka wizard laporan pemilik, klik Ekspor Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>File spreadsheet multi-tab (Summary, I&amp;E, Receipts, Balances, TB) terunduh</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Finance / Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>TC-66</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>rental_management_financial_report</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Generator Nomor Virtual Account &amp; QRIS</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Pilih bank VA pada kontrak, buka invoice tagihan sewa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Nomor VA (prefix+digits) dan blok QRIS tertera di form invoice &amp; portal</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Tenant / Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>TC-67</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>rental_management_financial_report</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Surat Izin Kerja (SIK) Renovasi / SIK PDF</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Buat SIK baru, pilih kontraktor &amp; jam kerja malam/hot work, setujui &amp; cetak PDF</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Dokumen SIK PDF bertandatangan 3 pihak terbit rapi</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>BM / Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>TC-68</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>rental_management_gto_meter</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Tarif Beban Puncak Listrik PLN (WBP/LWBP)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Centang tarif ganda pada meteran listrik, input stand WBP &amp; LWBP</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Konsumsi &amp; biaya WBP + LWBP terhitung akurat pada invoice</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Engineering / MEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>TC-69</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>rental_management_portal</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Rating Kepuasan CSAT pada Portal Maintenance</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Buka tiket maintenance selesai di portal /my/maintenance/&lt;id&gt;, beri rating &amp; ulasan</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Rating bintang &amp; feedback tersimpan dan tercatat di Chatter backend</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Tenant / CS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add Phase 7 enterprise enhancements (Parking RFID, 12M Cash Flow, Facility Booking, FX Lease Rates, Lease Amendment)
- Add Tenant Parking Pass (property.parking.pass) RFID registration, quotas, and printable PDF
- Add 12-Month Rolling Cash Flow Projection wizard (PDF & multi-tab Excel export)
- Add Function Room & Facility Booking (property.facility.booking) with conflict check & auto-invoicing
- Add Foreign Currency (USD/SGD) Lease handling with official KMK & BI exchange rates in CORETAX
- Add Lease Amendment & Rent Review Tracking (property.tenancy.amendment) with contract update & printable PDF
- Update User Guide (25 Chapters) and UAT Tracker (78 Test Cases)
</commit_message>
<xml_diff>
--- a/Rental Property Management - Odoo 19 Custom Addon/docs/UAT_Tracker_Custom_Modules.xlsx
+++ b/Rental Property Management - Odoo 19 Custom Addon/docs/UAT_Tracker_Custom_Modules.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4494,6 +4494,191 @@
       <c r="G100" t="inlineStr">
         <is>
           <t>Tenant / CS</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>TC-74</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>rental_management_parking</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Manajemen Pass Parkir Langganan &amp; RFID Kendaraan</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Daftarkan plat nomor kendaraan tenant, pilih jatah kuota gratis vs berbayar, cetak PDF</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Formulir pendaftaran &amp; kartu pass parkir PDF terbit dengan barcode/RFID</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Parking / BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>TC-75</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>rental_management_financial_report</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Proyeksi Arus Kas Bergulir 12 Bulan (PDF &amp; Excel)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Buka wizard proyeksi arus kas, pilih bulan awal, cetak PDF &amp; ekspor Excel</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Laporan arus kas 12 bulan (Inflows, Outflows, Net &amp; Cumulative) terbit akurat</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>CFO / Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>TC-76</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>rental_management_financial_report</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Pemesanan Fasilitas &amp; Ruang Rapat (Meeting Room)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Pilih fasilitas meeting room/ballroom, pilih sesi waktu, konfirmasi &amp; terbitkan invoice</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Validasi double-booking aktif dan invoice sewa + deposit kebersihan otomatis terbit</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Tenant / BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>TC-77</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>rental_management_coretax</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Kontrak Sewa Valas (USD/SGD) &amp; Kurs Pajak KMK/BI</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Centang sewa valas pada invoice, input nominal USD dan kurs KMK/BI</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Konversi DPP IDR dan e-Faktur CORETAX otomatis tersinkronisasi nilai Rupiah</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Tax / Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>TC-78</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>rental_management_rent_escalation</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Adendum Kontrak Sewa &amp; Audit Trail Perubahan</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Buat adendum perubahan tarif/tanggal sewa, setujui &amp; terapkan ke kontrak, cetak PDF</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Nilai kontrak induk otomatis terupdate dan dokumen Surat Adendum PDF tercetak rapi</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Legal / Leasing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add Phase 8 enterprise features (MEP Asset Checklist, GTO True-Up, Move-Out Clearance, IoT Smart Meter)
- Add MEP Equipment Asset & Mobile Technician Inspection Log (property.mep.asset)
- Add Annual GTO Turnover Rent True-Up Settlement wizard with auto invoice & PDF report
- Add 4-Division Tenant Move-Out Clearance Workflow (property.tenant.clearance) with deposit return PDF
- Add Smart Meter IoT REST Webhook Endpoint (/api/v1/meter/iot_reading)
- Update SOP User Guide (29 Chapters) and UAT Tracker (82 Test Cases)
</commit_message>
<xml_diff>
--- a/Rental Property Management - Odoo 19 Custom Addon/docs/UAT_Tracker_Custom_Modules.xlsx
+++ b/Rental Property Management - Odoo 19 Custom Addon/docs/UAT_Tracker_Custom_Modules.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4679,6 +4679,154 @@
       <c r="G105" t="inlineStr">
         <is>
           <t>Legal / Leasing</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>TC-79</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>rental_management_maintenance</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Manajemen Aset MEP &amp; Checklist Lapangan Teknisi</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Daftarkan alat MEP (genset/chiller), input log checklist harian, periksa status alert</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Log inspeksi tersimpan dan otomatis memicu warning alert bila status abnormal</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Engineering / MEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>TC-80</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>rental_management_gto_meter</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Rekonsiliasi Omzet Tahunan (GTO True-Up Settlement)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Input omzet audit tenant, hitung selisih bagi hasil omzet vs MGR, buat faktur penyesuaian</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Perhitungan selisih kekurangan omzet akurat dan faktur penyesuaian otomatis terbit</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Commercial / BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>TC-81</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>rental_management_financial_report</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Surat Bebas Kewajiban (Move-Out Clearance Workflow)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Buka form clearance, setujui sign-off 4 divisi, hitung pengembalian deposit, cetak PDF</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Surat Bebas Kewajiban &amp; Berita Acara Pengembalian Deposit PDF terbit resmi</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>BM / Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>TC-82</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>rental_management_gto_meter</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Integrasi API Smart Meter IoT (Listrik &amp; Air Digital)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Kirim POST request JSON payload ke /api/v1/meter/iot_reading</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Angka meteran terupdate otomatis tanpa input manual</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>IT / Engineering</t>
         </is>
       </c>
     </row>

</xml_diff>